<commit_message>
remove 'C1' mock for ldap and get back FG99
</commit_message>
<xml_diff>
--- a/assets/raw-data/biospecimen/test_bioproben.xlsx
+++ b/assets/raw-data/biospecimen/test_bioproben.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HesseE\mex-extractors\assets\raw-data\biospecimen\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esinsj\code\mex-extractors\assets\raw-data\biospecimen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354591A6-9D06-4C48-9836-C1B4890CFD8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E3FE32-FC4B-451E-889E-81330E2C3334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,8 +16,19 @@
     <sheet name="Probe1" sheetId="1" r:id="rId1"/>
     <sheet name="Probe2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -26,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="88">
   <si>
     <t>Probensammlung</t>
   </si>
@@ -286,7 +297,10 @@
     <t>testverwandedoi2</t>
   </si>
   <si>
-    <t>C1</t>
+    <t>PRNT</t>
+  </si>
+  <si>
+    <t>PARENT Dept.</t>
   </si>
 </sst>
 </file>
@@ -585,7 +599,7 @@
         <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>